<commit_message>
implementacion de flujo de aperturas, cierres y arqueos de caja
</commit_message>
<xml_diff>
--- a/public/TempReportsPage.xlsx
+++ b/public/TempReportsPage.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\amedina\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MANTUN PC\Documents\sistema_taller\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA827ACD-5DB0-4C3F-B1DF-C70CB51CD426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C3AAC5-4BC3-4406-BC11-816D972F6E62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{0415A6F6-D41A-436A-99D5-84249A168384}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0415A6F6-D41A-436A-99D5-84249A168384}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$G$61</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Hoja1!$A$1:$G$59</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -70,26 +69,18 @@
     <t>Hasta:</t>
   </si>
   <si>
-    <t>TOTALES</t>
-  </si>
-  <si>
-    <t>FIN DE PAGINA</t>
+    <t>Consolidado de Ventas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generado el: </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -116,10 +107,12 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="22"/>
-      <color theme="0" tint="-0.14999847407452621"/>
-      <name val="Arial Black"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -136,7 +129,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -159,40 +152,25 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -511,7 +489,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A3:G13"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" customWidth="1"/>
@@ -523,107 +501,105 @@
     <col min="7" max="7" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2" t="s">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="2"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+    <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+      <c r="D8" s="4"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+      <c r="D10" s="4"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
+      <c r="A13" s="3"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A10:G12"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="176" scale="74" fitToHeight="0" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>

</xml_diff>